<commit_message>
Implement incremental delta scraping with early stopping
</commit_message>
<xml_diff>
--- a/EXECUTIVE_TEAM_AUDIT_REPORT_15_Sep_2026.xlsx
+++ b/EXECUTIVE_TEAM_AUDIT_REPORT_15_Sep_2026.xlsx
@@ -532,14 +532,14 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="C3" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>66.7%</t>
         </is>
       </c>
     </row>
@@ -568,14 +568,14 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>60.0%</t>
         </is>
       </c>
     </row>
@@ -646,7 +646,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>25.0%</t>
+          <t>20.0%</t>
         </is>
       </c>
     </row>
@@ -657,19 +657,19 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C3" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="C3" s="2" t="n">
-        <v>2</v>
-      </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>66.7%</t>
+          <t>75.0%</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>75.0%</t>
+          <t>80.0%</t>
         </is>
       </c>
     </row>
@@ -731,13 +731,13 @@
         <v>0</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3">
@@ -769,13 +769,13 @@
         <v>1</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D4" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -789,11 +789,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX5"/>
+  <dimension ref="A1:AX6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="23" customWidth="1" min="2" max="2"/>
     <col width="35" customWidth="1" min="3" max="3"/>
     <col width="23" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
@@ -830,7 +830,7 @@
     <col width="26" customWidth="1" min="36" max="36"/>
     <col width="17" customWidth="1" min="37" max="37"/>
     <col width="18" customWidth="1" min="38" max="38"/>
-    <col width="23" customWidth="1" min="39" max="39"/>
+    <col width="20" customWidth="1" min="39" max="39"/>
     <col width="28" customWidth="1" min="40" max="40"/>
     <col width="27" customWidth="1" min="41" max="41"/>
     <col width="12" customWidth="1" min="42" max="42"/>
@@ -1163,10 +1163,8 @@
           <t>Chandramani Chaudhary</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr">
-        <is>
-          <t>9768922502</t>
-        </is>
+      <c r="O2" s="2" t="n">
+        <v>9768922502</v>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
@@ -1205,10 +1203,8 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="Y2" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="Y2" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1246,19 +1242,17 @@
           <t>Fiber wire breakage suspect</t>
         </is>
       </c>
-      <c r="AH2" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="AH2" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="AI2" s="2" t="inlineStr">
         <is>
-          <t>00:00 hour</t>
+          <t>00:52 hour</t>
         </is>
       </c>
       <c r="AJ2" s="2" t="inlineStr">
         <is>
-          <t>00:00 hour / 00:00 hour</t>
+          <t>23:08 hour / 00:00 hour</t>
         </is>
       </c>
       <c r="AK2" s="2" t="inlineStr"/>
@@ -1272,25 +1266,21 @@
           <t>Chandramani Tharu</t>
         </is>
       </c>
-      <c r="AN2" s="2" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="AN2" s="2" t="n">
+        <v>6</v>
       </c>
       <c r="AO2" s="2" t="inlineStr">
         <is>
           <t>CDB314</t>
         </is>
       </c>
-      <c r="AP2" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="AP2" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="AQ2" s="2" t="inlineStr"/>
       <c r="AR2" s="2" t="inlineStr">
         <is>
-          <t>Case : fiber issue   has been updated by Chandramani Tharu</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="AS2" s="2" t="inlineStr">
@@ -1378,7 +1368,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
@@ -1391,10 +1381,8 @@
           <t>Sudharna Byanjankar</t>
         </is>
       </c>
-      <c r="O3" s="2" t="inlineStr">
-        <is>
-          <t>9851316119</t>
-        </is>
+      <c r="O3" s="2" t="n">
+        <v>9851316119</v>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
@@ -1421,7 +1409,7 @@
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>15 Sep 2026 09:04:22 AM</t>
+          <t>15 Sep 2026 10:39:23 AM</t>
         </is>
       </c>
       <c r="X3" s="2" t="inlineStr">
@@ -1429,10 +1417,8 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="Y3" s="2" t="inlineStr">
-        <is>
-          <t>27.67154</t>
-        </is>
+      <c r="Y3" s="2" t="n">
+        <v>27.67154</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1441,7 +1427,7 @@
       </c>
       <c r="AA3" s="2" t="inlineStr">
         <is>
-          <t>Layer 1-User</t>
+          <t>Layer 1-</t>
         </is>
       </c>
       <c r="AB3" s="2" t="inlineStr">
@@ -1485,43 +1471,39 @@
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>Shashikant Chaudhary</t>
-        </is>
-      </c>
-      <c r="AN3" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+          <t>Rahul Chaudhary</t>
+        </is>
+      </c>
+      <c r="AN3" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="AO3" s="2" t="inlineStr">
         <is>
           <t>2,6</t>
         </is>
       </c>
-      <c r="AP3" s="2" t="inlineStr">
-        <is>
-          <t>85.33876</t>
-        </is>
+      <c r="AP3" s="2" t="n">
+        <v>85.33875999999999</v>
       </c>
       <c r="AQ3" s="2" t="inlineStr"/>
       <c r="AR3" s="2" t="inlineStr">
         <is>
-          <t>Case : WiFi 6  has been updated by Shashikant Chaudhary</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="AS3" s="2" t="inlineStr">
         <is>
-          <t>0m</t>
+          <t>1h 35m</t>
         </is>
       </c>
       <c r="AT3" s="2" t="inlineStr">
         <is>
-          <t>11h 11m</t>
+          <t>12h 46m</t>
         </is>
       </c>
       <c r="AU3" s="2" t="inlineStr">
         <is>
-          <t>Completed (Completed)</t>
+          <t>Completed (Closed)</t>
         </is>
       </c>
       <c r="AV3" s="2" t="inlineStr">
@@ -1548,7 +1530,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>15 Sep 2026 9:24 AM</t>
+          <t>15 Sep 2026 10:55 AM</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -1574,7 +1556,7 @@
       <c r="G4" s="2" t="inlineStr"/>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Case : wifi 6  has been updated by Sabin Giri</t>
+          <t>Case : wifi 6   has been updated by Sabin Giri</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -1584,32 +1566,32 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>TKT1334065</t>
+          <t>TKT1333510</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>Saradha Panta</t>
+          <t>Kabiraj Limbu</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>Phone</t>
+          <t>None</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>Saradha Panta</t>
+          <t>Kabiraj Limbu</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>9851322004</t>
+          <t>9825986033</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -1620,24 +1602,24 @@
       <c r="Q4" s="2" t="inlineStr"/>
       <c r="R4" s="2" t="inlineStr">
         <is>
-          <t>15 Sep 2026 07:57:11 AM</t>
+          <t>15 Sep 2026 10:55:56 AM</t>
         </is>
       </c>
       <c r="S4" s="2" t="inlineStr"/>
       <c r="T4" s="2" t="inlineStr"/>
       <c r="U4" s="2" t="inlineStr">
         <is>
-          <t>9851322004</t>
+          <t>BKT9825986033</t>
         </is>
       </c>
       <c r="V4" s="2" t="inlineStr">
         <is>
-          <t>15 Sep 2026 07:57:11 AM</t>
+          <t>14 Sep 2026 01:24:32 PM</t>
         </is>
       </c>
       <c r="W4" s="2" t="inlineStr">
         <is>
-          <t>15 Sep 2026 09:38:08 AM</t>
+          <t>15 Sep 2026 10:55:56 AM</t>
         </is>
       </c>
       <c r="X4" s="2" t="inlineStr">
@@ -1645,11 +1627,7 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="Y4" s="2" t="inlineStr">
-        <is>
-          <t>27.71579</t>
-        </is>
-      </c>
+      <c r="Y4" s="2" t="inlineStr"/>
       <c r="Z4" s="2" t="inlineStr">
         <is>
           <t>General / Other Issues</t>
@@ -1662,7 +1640,7 @@
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
-          <t>Laxman Koirala</t>
+          <t>L1  Support</t>
         </is>
       </c>
       <c r="AC4" s="2" t="inlineStr">
@@ -1673,12 +1651,12 @@
       <c r="AD4" s="2" t="inlineStr"/>
       <c r="AE4" s="2" t="inlineStr">
         <is>
-          <t>Sarveshwor Mahadev Temple, Nayabasti, Bagmati, Central, Nepal</t>
+          <t>Kageshwori Manohara Municipality Ward No.7 office - Local government office P92M+XX3 Kageshwori Mano</t>
         </is>
       </c>
       <c r="AF4" s="2" t="inlineStr">
         <is>
-          <t>workcgnet@gmail.com</t>
+          <t>test@test.com</t>
         </is>
       </c>
       <c r="AG4" s="2" t="inlineStr">
@@ -1687,17 +1665,21 @@
         </is>
       </c>
       <c r="AH4" s="2" t="inlineStr"/>
-      <c r="AI4" s="2" t="inlineStr"/>
+      <c r="AI4" s="2" t="inlineStr">
+        <is>
+          <t>07:31 hour</t>
+        </is>
+      </c>
       <c r="AJ4" s="2" t="inlineStr"/>
       <c r="AK4" s="2" t="inlineStr"/>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>Nisha Joshi</t>
+          <t>Kusum Gurung</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>Monali Lohani</t>
+          <t>Sabin Giri</t>
         </is>
       </c>
       <c r="AN4" s="2" t="inlineStr">
@@ -1707,38 +1689,34 @@
       </c>
       <c r="AO4" s="2" t="inlineStr">
         <is>
-          <t>L31-6</t>
-        </is>
-      </c>
-      <c r="AP4" s="2" t="inlineStr">
-        <is>
-          <t>85.36397</t>
-        </is>
-      </c>
+          <t>L37-1</t>
+        </is>
+      </c>
+      <c r="AP4" s="2" t="inlineStr"/>
       <c r="AQ4" s="2" t="inlineStr"/>
       <c r="AR4" s="2" t="inlineStr">
         <is>
-          <t>Case : wifi 6  has been updated by Sabin Giri</t>
+          <t>Case : wifi 6   has been updated by Sabin Giri</t>
         </is>
       </c>
       <c r="AS4" s="2" t="inlineStr">
         <is>
-          <t>1h 40m</t>
+          <t>0m</t>
         </is>
       </c>
       <c r="AT4" s="2" t="inlineStr">
         <is>
-          <t>1h 40m</t>
+          <t>21h 31m</t>
         </is>
       </c>
       <c r="AU4" s="2" t="inlineStr">
         <is>
-          <t>Other / In Progress (In Progress)</t>
+          <t>Completed (Completed)</t>
         </is>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>Case : wifi 6  has been updated by Sabin Giri</t>
+          <t>Case : wifi 6   has been updated by Sabin Giri</t>
         </is>
       </c>
       <c r="AW4" s="2" t="inlineStr">
@@ -1760,7 +1738,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>15 Sep 2026 8:51 AM</t>
+          <t>15 Sep 2026 9:24 AM</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -1786,7 +1764,7 @@
       <c r="G5" s="2" t="inlineStr"/>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Case : wifi 6   has been updated by Sabin Giri</t>
+          <t>Case : wifi 6  has been updated by Sabin Giri</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -1796,17 +1774,17 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>TKT1333787</t>
+          <t>TKT1334065</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>Ganesh bahadur dhakal</t>
+          <t>Saradha Panta</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
@@ -1816,12 +1794,12 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>Ganesh bahadur dhakal</t>
+          <t>Saradha Panta</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>9841051986</t>
+          <t>9851322004</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -1832,24 +1810,24 @@
       <c r="Q5" s="2" t="inlineStr"/>
       <c r="R5" s="2" t="inlineStr">
         <is>
-          <t>15 Sep 2026 08:51:57 AM</t>
+          <t>15 Sep 2026 07:57:11 AM</t>
         </is>
       </c>
       <c r="S5" s="2" t="inlineStr"/>
       <c r="T5" s="2" t="inlineStr"/>
       <c r="U5" s="2" t="inlineStr">
         <is>
-          <t>9841051986</t>
+          <t>9851322004</t>
         </is>
       </c>
       <c r="V5" s="2" t="inlineStr">
         <is>
-          <t>14 Sep 2026 05:06:15 PM</t>
+          <t>15 Sep 2026 07:57:11 AM</t>
         </is>
       </c>
       <c r="W5" s="2" t="inlineStr">
         <is>
-          <t>15 Sep 2026 08:51:57 AM</t>
+          <t>15 Sep 2026 09:38:08 AM</t>
         </is>
       </c>
       <c r="X5" s="2" t="inlineStr">
@@ -1857,7 +1835,11 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="Y5" s="2" t="inlineStr"/>
+      <c r="Y5" s="2" t="inlineStr">
+        <is>
+          <t>27.71579</t>
+        </is>
+      </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
           <t>General / Other Issues</t>
@@ -1870,7 +1852,7 @@
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
-          <t>L1  Support</t>
+          <t>Laxman Koirala</t>
         </is>
       </c>
       <c r="AC5" s="2" t="inlineStr">
@@ -1881,31 +1863,31 @@
       <c r="AD5" s="2" t="inlineStr"/>
       <c r="AE5" s="2" t="inlineStr">
         <is>
-          <t>Dhakchin dhoka the luga ghar, Bagmati, Central, Nepal</t>
-        </is>
-      </c>
-      <c r="AF5" s="2" t="inlineStr"/>
+          <t>Sarveshwor Mahadev Temple, Nayabasti, Bagmati, Central, Nepal</t>
+        </is>
+      </c>
+      <c r="AF5" s="2" t="inlineStr">
+        <is>
+          <t>workcgnet@gmail.com</t>
+        </is>
+      </c>
       <c r="AG5" s="2" t="inlineStr">
         <is>
           <t>Router Upgrade  Wi-Fi 6</t>
         </is>
       </c>
       <c r="AH5" s="2" t="inlineStr"/>
-      <c r="AI5" s="2" t="inlineStr">
-        <is>
-          <t>02:54 hour</t>
-        </is>
-      </c>
+      <c r="AI5" s="2" t="inlineStr"/>
       <c r="AJ5" s="2" t="inlineStr"/>
       <c r="AK5" s="2" t="inlineStr"/>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>Aakash Shah</t>
+          <t>Nisha Joshi</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>Sabin Giri</t>
+          <t>Monali Lohani</t>
         </is>
       </c>
       <c r="AN5" s="2" t="inlineStr">
@@ -1915,42 +1897,250 @@
       </c>
       <c r="AO5" s="2" t="inlineStr">
         <is>
-          <t>L15-2</t>
-        </is>
-      </c>
-      <c r="AP5" s="2" t="inlineStr"/>
+          <t>L31-6</t>
+        </is>
+      </c>
+      <c r="AP5" s="2" t="inlineStr">
+        <is>
+          <t>85.36397</t>
+        </is>
+      </c>
       <c r="AQ5" s="2" t="inlineStr"/>
       <c r="AR5" s="2" t="inlineStr">
         <is>
+          <t>Case : wifi 6  has been updated by Sabin Giri</t>
+        </is>
+      </c>
+      <c r="AS5" s="2" t="inlineStr">
+        <is>
+          <t>1h 40m</t>
+        </is>
+      </c>
+      <c r="AT5" s="2" t="inlineStr">
+        <is>
+          <t>1h 40m</t>
+        </is>
+      </c>
+      <c r="AU5" s="2" t="inlineStr">
+        <is>
+          <t>Other / In Progress (In Progress)</t>
+        </is>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>Case : wifi 6  has been updated by Sabin Giri</t>
+        </is>
+      </c>
+      <c r="AW5" s="2" t="inlineStr">
+        <is>
+          <t>WiFi 6 Upgrade</t>
+        </is>
+      </c>
+      <c r="AX5" s="2" t="inlineStr">
+        <is>
+          <t>Sabin Giri</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Sabin Giri</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>15 Sep 2026 8:51 AM</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>WGnmUJF06LTlUriJ5DeDBQ==</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Sabin Giri</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Case</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
           <t>Case : wifi 6   has been updated by Sabin Giri</t>
         </is>
       </c>
-      <c r="AS5" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>wifi 6</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>TKT1333787</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>Ganesh bahadur dhakal</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>Ganesh bahadur dhakal</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>9841051986</t>
+        </is>
+      </c>
+      <c r="P6" s="2" t="inlineStr">
+        <is>
+          <t>General / Other Issues</t>
+        </is>
+      </c>
+      <c r="Q6" s="2" t="inlineStr"/>
+      <c r="R6" s="2" t="inlineStr">
+        <is>
+          <t>15 Sep 2026 08:51:57 AM</t>
+        </is>
+      </c>
+      <c r="S6" s="2" t="inlineStr"/>
+      <c r="T6" s="2" t="inlineStr"/>
+      <c r="U6" s="2" t="inlineStr">
+        <is>
+          <t>9841051986</t>
+        </is>
+      </c>
+      <c r="V6" s="2" t="inlineStr">
+        <is>
+          <t>14 Sep 2026 05:06:15 PM</t>
+        </is>
+      </c>
+      <c r="W6" s="2" t="inlineStr">
+        <is>
+          <t>15 Sep 2026 08:51:57 AM</t>
+        </is>
+      </c>
+      <c r="X6" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="Y6" s="2" t="inlineStr"/>
+      <c r="Z6" s="2" t="inlineStr">
+        <is>
+          <t>General / Other Issues</t>
+        </is>
+      </c>
+      <c r="AA6" s="2" t="inlineStr">
+        <is>
+          <t>Layer 1-User</t>
+        </is>
+      </c>
+      <c r="AB6" s="2" t="inlineStr">
+        <is>
+          <t>L1  Support</t>
+        </is>
+      </c>
+      <c r="AC6" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="AD6" s="2" t="inlineStr"/>
+      <c r="AE6" s="2" t="inlineStr">
+        <is>
+          <t>Dhakchin dhoka the luga ghar, Bagmati, Central, Nepal</t>
+        </is>
+      </c>
+      <c r="AF6" s="2" t="inlineStr"/>
+      <c r="AG6" s="2" t="inlineStr">
+        <is>
+          <t>Router Upgrade  Wi-Fi 6</t>
+        </is>
+      </c>
+      <c r="AH6" s="2" t="inlineStr"/>
+      <c r="AI6" s="2" t="inlineStr">
+        <is>
+          <t>02:54 hour</t>
+        </is>
+      </c>
+      <c r="AJ6" s="2" t="inlineStr"/>
+      <c r="AK6" s="2" t="inlineStr"/>
+      <c r="AL6" s="2" t="inlineStr">
+        <is>
+          <t>Aakash Shah</t>
+        </is>
+      </c>
+      <c r="AM6" s="2" t="inlineStr">
+        <is>
+          <t>Sabin Giri</t>
+        </is>
+      </c>
+      <c r="AN6" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="AO6" s="2" t="inlineStr">
+        <is>
+          <t>L15-2</t>
+        </is>
+      </c>
+      <c r="AP6" s="2" t="inlineStr"/>
+      <c r="AQ6" s="2" t="inlineStr"/>
+      <c r="AR6" s="2" t="inlineStr">
+        <is>
+          <t>Case : wifi 6   has been updated by Sabin Giri</t>
+        </is>
+      </c>
+      <c r="AS6" s="2" t="inlineStr">
         <is>
           <t>0m</t>
         </is>
       </c>
-      <c r="AT5" s="2" t="inlineStr">
+      <c r="AT6" s="2" t="inlineStr">
         <is>
           <t>15h 45m</t>
         </is>
       </c>
-      <c r="AU5" s="2" t="inlineStr">
+      <c r="AU6" s="2" t="inlineStr">
         <is>
           <t>Completed (Completed)</t>
         </is>
       </c>
-      <c r="AV5" s="2" t="inlineStr">
+      <c r="AV6" s="2" t="inlineStr">
         <is>
           <t>Case : wifi 6   has been updated by Sabin Giri</t>
         </is>
       </c>
-      <c r="AW5" s="2" t="inlineStr">
+      <c r="AW6" s="2" t="inlineStr">
         <is>
           <t>WiFi 6 Upgrade</t>
         </is>
       </c>
-      <c r="AX5" s="2" t="inlineStr">
+      <c r="AX6" s="2" t="inlineStr">
         <is>
           <t>Sabin Giri</t>
         </is>

</xml_diff>

<commit_message>
Display full technician matrix with all 8 team members and add dedicated technician and category summary tables
</commit_message>
<xml_diff>
--- a/EXECUTIVE_TEAM_AUDIT_REPORT_15_Sep_2026.xlsx
+++ b/EXECUTIVE_TEAM_AUDIT_REPORT_15_Sep_2026.xlsx
@@ -476,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -510,11 +510,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Chandramani Tharu</t>
+          <t>Ajit Shrestha</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C2" s="2" t="n">
         <v>0</v>
@@ -528,52 +528,142 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Sabin Giri</t>
+          <t>Chandramani Tharu</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>66.7%</t>
+          <t>0.0%</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Shashikant Chaudhary</t>
+          <t>Om Neupane</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>0.0%</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Rajesh Maharjan</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Sabin Giri</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>66.7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Sanjeev Giri</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Shashikant Chaudhary</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Sunil Chaudhary</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>👥 GRAND TOTAL (ALL TEAM)</t>
         </is>
       </c>
-      <c r="B5" s="3" t="n">
+      <c r="B10" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="C5" s="3" t="n">
+      <c r="C10" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>60.0%</t>
         </is>
@@ -684,14 +774,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="23" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="23" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -702,20 +797,45 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Ajit Shrestha</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Chandramani Tharu</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Om Neupane</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Rajesh Maharjan</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Sabin Giri</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Sanjeev Giri</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Shashikant Chaudhary</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Sunil Chaudhary</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Grand Total</t>
         </is>
@@ -731,12 +851,27 @@
         <v>0</v>
       </c>
       <c r="C2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="D2" s="2" t="n">
+      <c r="G2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E2" s="4" t="n">
+      <c r="I2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" s="4" t="n">
         <v>4</v>
       </c>
     </row>
@@ -747,15 +882,30 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C3" s="2" t="n">
-        <v>0</v>
-      </c>
       <c r="D3" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="E3" s="4" t="n">
+      <c r="E3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" s="4" t="n">
         <v>1</v>
       </c>
     </row>
@@ -766,15 +916,30 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="C4" s="3" t="n">
+      <c r="D4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="D4" s="3" t="n">
+      <c r="G4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="E4" s="3" t="n">
+      <c r="I4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="3" t="n">
         <v>5</v>
       </c>
     </row>
@@ -789,7 +954,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX6"/>
+  <dimension ref="A1:AY6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -842,6 +1007,7 @@
     <col width="45" customWidth="1" min="48" max="48"/>
     <col width="25" customWidth="1" min="49" max="49"/>
     <col width="23" customWidth="1" min="50" max="50"/>
+    <col width="16" customWidth="1" min="51" max="51"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1095,6 +1261,11 @@
           <t>Employee Name</t>
         </is>
       </c>
+      <c r="AY1" s="1" t="inlineStr">
+        <is>
+          <t>Is_Solved_Val</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1278,11 +1449,7 @@
         <v>0</v>
       </c>
       <c r="AQ2" s="2" t="inlineStr"/>
-      <c r="AR2" s="2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="AR2" s="2" t="inlineStr"/>
       <c r="AS2" s="2" t="inlineStr">
         <is>
           <t>7m</t>
@@ -1312,6 +1479,9 @@
         <is>
           <t>Chandramani Tharu</t>
         </is>
+      </c>
+      <c r="AY2" s="2" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -1486,11 +1656,7 @@
         <v>85.33875999999999</v>
       </c>
       <c r="AQ3" s="2" t="inlineStr"/>
-      <c r="AR3" s="2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="AR3" s="2" t="inlineStr"/>
       <c r="AS3" s="2" t="inlineStr">
         <is>
           <t>1h 35m</t>
@@ -1520,6 +1686,9 @@
         <is>
           <t>Shashikant Chaudhary</t>
         </is>
+      </c>
+      <c r="AY3" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -1579,20 +1748,14 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="M4" s="2" t="inlineStr"/>
       <c r="N4" s="2" t="inlineStr">
         <is>
           <t>Kabiraj Limbu</t>
         </is>
       </c>
-      <c r="O4" s="2" t="inlineStr">
-        <is>
-          <t>9825986033</t>
-        </is>
+      <c r="O4" s="2" t="n">
+        <v>9825986033</v>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
@@ -1682,10 +1845,8 @@
           <t>Sabin Giri</t>
         </is>
       </c>
-      <c r="AN4" s="2" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="AN4" s="2" t="n">
+        <v>6</v>
       </c>
       <c r="AO4" s="2" t="inlineStr">
         <is>
@@ -1729,6 +1890,9 @@
           <t>Sabin Giri</t>
         </is>
       </c>
+      <c r="AY4" s="2" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1797,10 +1961,8 @@
           <t>Saradha Panta</t>
         </is>
       </c>
-      <c r="O5" s="2" t="inlineStr">
-        <is>
-          <t>9851322004</t>
-        </is>
+      <c r="O5" s="2" t="n">
+        <v>9851322004</v>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
@@ -1835,10 +1997,8 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="Y5" s="2" t="inlineStr">
-        <is>
-          <t>27.71579</t>
-        </is>
+      <c r="Y5" s="2" t="n">
+        <v>27.71579</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1890,20 +2050,16 @@
           <t>Monali Lohani</t>
         </is>
       </c>
-      <c r="AN5" s="2" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="AN5" s="2" t="n">
+        <v>6</v>
       </c>
       <c r="AO5" s="2" t="inlineStr">
         <is>
           <t>L31-6</t>
         </is>
       </c>
-      <c r="AP5" s="2" t="inlineStr">
-        <is>
-          <t>85.36397</t>
-        </is>
+      <c r="AP5" s="2" t="n">
+        <v>85.36396999999999</v>
       </c>
       <c r="AQ5" s="2" t="inlineStr"/>
       <c r="AR5" s="2" t="inlineStr">
@@ -1940,6 +2096,9 @@
         <is>
           <t>Sabin Giri</t>
         </is>
+      </c>
+      <c r="AY5" s="2" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -2009,10 +2168,8 @@
           <t>Ganesh bahadur dhakal</t>
         </is>
       </c>
-      <c r="O6" s="2" t="inlineStr">
-        <is>
-          <t>9841051986</t>
-        </is>
+      <c r="O6" s="2" t="n">
+        <v>9841051986</v>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
@@ -2098,10 +2255,8 @@
           <t>Sabin Giri</t>
         </is>
       </c>
-      <c r="AN6" s="2" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="AN6" s="2" t="n">
+        <v>6</v>
       </c>
       <c r="AO6" s="2" t="inlineStr">
         <is>
@@ -2144,6 +2299,9 @@
         <is>
           <t>Sabin Giri</t>
         </is>
+      </c>
+      <c r="AY6" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>